<commit_message>
Update Status of project
</commit_message>
<xml_diff>
--- a/Documentation/Dictionary.xlsx
+++ b/Documentation/Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/562f170528f46325/My Documents/GitHub/ge-smarttemp/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="220" documentId="8_{41BC8FF7-AB83-E74E-8837-E1FCC09A0C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE684163-11BD-D449-9B74-99FCCC20922E}"/>
+  <xr:revisionPtr revIDLastSave="223" documentId="8_{41BC8FF7-AB83-E74E-8837-E1FCC09A0C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4571A8D2-673C-594A-86B9-DBD34C81A19A}"/>
   <bookViews>
-    <workbookView xWindow="3920" yWindow="10800" windowWidth="28780" windowHeight="16280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="26800" yWindow="2480" windowWidth="28800" windowHeight="16300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dictionary" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
     </textPr>
   </connection>
   <connection id="2" xr16:uid="{C561AA97-0CB1-CE4B-B8A1-CEF82942D0E5}" name="Lounge.pair_key" type="6" refreshedVersion="8" background="1" saveData="1">
-    <textPr codePage="10000" sourceFile="/Users/robert/Library/CloudStorage/OneDrive-Personal/Desktop/Lounge.pair_key.json">
+    <textPr sourceFile="/Users/robert/Library/CloudStorage/OneDrive-Personal/Desktop/Lounge.pair_key.json">
       <textFields count="4">
         <textField/>
         <textField/>
@@ -675,6 +675,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1360,7 +1364,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57E9865F-8FFC-D44B-8B68-BB05D4233726}">
-  <dimension ref="A1:F174"/>
+  <dimension ref="A1:I180"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="1.6640625" bestFit="1" customWidth="1"/>
@@ -1369,6 +1373,7 @@
     <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="2.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.15">
@@ -2662,6 +2667,22 @@
     <row r="174" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A174" t="s">
         <v>111</v>
+      </c>
+    </row>
+    <row r="178" spans="9:9" x14ac:dyDescent="0.15">
+      <c r="I178">
+        <v>1767619818</v>
+      </c>
+    </row>
+    <row r="179" spans="9:9" x14ac:dyDescent="0.15">
+      <c r="I179">
+        <v>1767616218</v>
+      </c>
+    </row>
+    <row r="180" spans="9:9" x14ac:dyDescent="0.15">
+      <c r="I180">
+        <f>I179-I178</f>
+        <v>-3600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean up of Hub code
</commit_message>
<xml_diff>
--- a/Documentation/Dictionary.xlsx
+++ b/Documentation/Dictionary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/562f170528f46325/My Documents/GitHub/ge-smarttemp/Documentation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/562f170528f46325/My Documents/GitHub/ha-smarttemp/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="223" documentId="8_{41BC8FF7-AB83-E74E-8837-E1FCC09A0C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4571A8D2-673C-594A-86B9-DBD34C81A19A}"/>
   <bookViews>
-    <workbookView xWindow="26800" yWindow="2480" windowWidth="28800" windowHeight="16300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34780" yWindow="18140" windowWidth="28800" windowHeight="16300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dictionary" sheetId="1" r:id="rId1"/>

</xml_diff>